<commit_message>
Save point: Liane Jamason full SEO audit complete
All research, deliverables, and client files finalized:
- audit-data.json populated with real data from 6 research agents
- Excel workbook and PowerPoint regenerated from audit data
- Claude vs Codex review (Claude wins 141/160 vs 120/160)
- Verification report (approved with required actions)
- Grade: D+ — strong content assets, severe technical SEO gaps

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/liane-jamason/seo/reports/SEO-Audit-GamePlan.xlsx
+++ b/clients/liane-jamason/seo/reports/SEO-Audit-GamePlan.xlsx
@@ -413,7 +413,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SEO Audit: example.com</v>
+        <v>SEO Audit: lianejamason.com</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -430,7 +430,7 @@
         <v>Prepared For:</v>
       </c>
       <c r="B2" t="str">
-        <v>Client Name</v>
+        <v>Liane Jamason</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -444,7 +444,7 @@
         <v>Company:</v>
       </c>
       <c r="B3" t="str">
-        <v>Brokerage / Company Name</v>
+        <v>Corcoran Dwellings</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -458,7 +458,7 @@
         <v>Website:</v>
       </c>
       <c r="B4" t="str">
-        <v>https://www.example.com</v>
+        <v>https://www.lianejamason.com/</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -472,7 +472,7 @@
         <v>Platform:</v>
       </c>
       <c r="B5" t="str">
-        <v>Website Platform</v>
+        <v>WordPress (Genesis Framework / AgentPress theme)</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v>Audit Date:</v>
       </c>
       <c r="B6" t="str">
-        <v>March 1, 2026</v>
+        <v>April 8, 2026</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -542,7 +542,7 @@
         <v>1</v>
       </c>
       <c r="B11" t="str">
-        <v>Zero organic search visibility — Not found for any of 25 target keywords — potential clients cannot find this site through Google</v>
+        <v>Zero non-branded organic visibility — Ranks for only 2 of 25 target keywords — both branded queries. Zero ranking for any commercial keyword (luxury homes, waterfront homes, neighborhoods, agent intent)</v>
       </c>
       <c r="C11" t="str">
         <v>Critical</v>
@@ -556,13 +556,13 @@
         <v>2</v>
       </c>
       <c r="B12" t="str">
-        <v>Critically thin content — Far fewer pages than competitors; dead or nonexistent blog</v>
+        <v>Broken primary lead capture funnel — Market Analysis / home valuation form is non-rendering. Homepage CTA 'What's My Home Worth?' leads to a dead end. Seller conversion path is completely broken</v>
       </c>
       <c r="C12" t="str">
         <v>Critical</v>
       </c>
       <c r="D12" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
     </row>
     <row r="13">
@@ -570,13 +570,13 @@
         <v>3</v>
       </c>
       <c r="B13" t="str">
-        <v>No locally-focused content — Missing the #1 content type for local SEO in this industry</v>
+        <v>60%+ of core pages missing meta descriptions — Homepage, blog index, reviews, property search, active listings, sold listings, and most area pages have no meta descriptions. Google auto-generates poor snippets</v>
       </c>
       <c r="C13" t="str">
         <v>Critical</v>
       </c>
       <c r="D13" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
     </row>
     <row r="14">
@@ -584,13 +584,13 @@
         <v>4</v>
       </c>
       <c r="B14" t="str">
-        <v>Technical SEO errors — Broken pages, corrupted meta tags, missing schema markup, images without alt text</v>
+        <v>70-83% of images missing alt text — Hero images, professional headshot, press logos (Bay News 9, Tampa Bay Times, HuffPost), property photos, and blog featured images all lack alt text</v>
       </c>
       <c r="C14" t="str">
         <v>High</v>
       </c>
       <c r="D14" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="15">
@@ -598,13 +598,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="str">
-        <v>No lead capture on key pages — Highest-traffic pages have no forms, CTAs, or lead magnets</v>
+        <v>Broken sitemap and thin-page indexing — 7 attachment sitemaps feeding hundreds of thin media pages into Google's index. One broken sitemap returning 404. Crawl budget wasted on junk content</v>
       </c>
       <c r="C15" t="str">
         <v>High</v>
       </c>
       <c r="D15" t="str">
-        <v>Low-Medium</v>
+        <v>Low</v>
       </c>
     </row>
     <row r="17">
@@ -629,10 +629,10 @@
         <v>Metric</v>
       </c>
       <c r="B18" t="str">
-        <v>example.com</v>
+        <v>lianejamason.com</v>
       </c>
       <c r="C18" t="str">
-        <v>#1 Competitor (Competitor 1)</v>
+        <v>#1 Competitor (Avalon Group)</v>
       </c>
       <c r="D18" t="str">
         <v>Gap</v>
@@ -645,14 +645,14 @@
       <c r="A19" t="str">
         <v>Total Pages</v>
       </c>
-      <c r="B19">
-        <v>62</v>
-      </c>
-      <c r="C19">
-        <v>376</v>
+      <c r="B19" t="str">
+        <v>365+</v>
+      </c>
+      <c r="C19" t="str">
+        <v>287-1,100+</v>
       </c>
       <c r="D19" t="str">
-        <v>6x behind</v>
+        <v>Volume exists but technical issues prevent visibility</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -662,14 +662,14 @@
       <c r="A20" t="str">
         <v>Blog Posts</v>
       </c>
-      <c r="B20">
-        <v>5</v>
-      </c>
-      <c r="C20">
-        <v>33</v>
+      <c r="B20" t="str">
+        <v>287</v>
+      </c>
+      <c r="C20" t="str">
+        <v>10-235</v>
       </c>
       <c r="D20" t="str">
-        <v>Blog is dead</v>
+        <v>Leads most competitors in volume</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -677,16 +677,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Key Pages Depth</v>
+        <v>Neighborhood Pages</v>
       </c>
       <c r="B21" t="str">
-        <v>~200 words</v>
+        <v>15+</v>
       </c>
       <c r="C21" t="str">
-        <v>3,500+ words</v>
+        <v>7-50+</v>
       </c>
       <c r="D21" t="str">
-        <v>~20x gap per page</v>
+        <v>Mid-range; needs expansion + depth</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -697,13 +697,13 @@
         <v>Schema Markup</v>
       </c>
       <c r="B22" t="str">
-        <v>None</v>
+        <v>Moderate (basic types)</v>
       </c>
       <c r="C22" t="str">
-        <v>Yes (all pages)</v>
+        <v>Excellent (Eagan: AggregateRating, AggregateOffer, Service)</v>
       </c>
       <c r="D22" t="str">
-        <v>Critical missing feature</v>
+        <v>Missing review stars, FAQ, breadcrumbs</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -713,14 +713,14 @@
       <c r="A23" t="str">
         <v>Keywords Ranking (of 25)</v>
       </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>12</v>
+      <c r="B23" t="str">
+        <v>2 (branded only)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Up to 12 (Lipply Real Estate)</v>
       </c>
       <c r="D23" t="str">
-        <v>Zero visibility</v>
+        <v>Zero commercial visibility</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -728,16 +728,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>FAQ Sections</v>
+        <v>Homepage Meta Description</v>
       </c>
       <c r="B24" t="str">
-        <v>None</v>
+        <v>MISSING</v>
       </c>
       <c r="C24" t="str">
-        <v>Yes</v>
+        <v>Present (4 of 5 competitors)</v>
       </c>
       <c r="D24" t="str">
-        <v>Missing rich snippet opportunity</v>
+        <v>Critical missing element</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -752,7 +752,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F29"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -764,7 +764,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>KEYWORD RESEARCH: City, State (5 Keywords)</v>
+        <v>KEYWORD RESEARCH: St. Petersburg, FL (25 Keywords)</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -784,7 +784,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Keywords Tested: 5 | Client Rankings Found: 0 | Competitor 1 Rankings: 2</v>
+        <v>Keywords Tested: 25 | Client Rankings Found: 2 | Avalon Group Rankings: 7</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -813,10 +813,10 @@
         <v>Est. Volume</v>
       </c>
       <c r="D4" t="str">
-        <v>example.com</v>
+        <v>lianejamason.com</v>
       </c>
       <c r="E4" t="str">
-        <v>competitor1.com</v>
+        <v>avalongrouptampabay.com</v>
       </c>
       <c r="F4" t="str">
         <v>Top Organic Result</v>
@@ -827,19 +827,19 @@
         <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>primary keyword 1</v>
+        <v>Liane Jamason realtor St Petersburg FL</v>
       </c>
       <c r="C5" t="str">
-        <v>Very High</v>
+        <v>Low</v>
       </c>
       <c r="D5" t="str">
-        <v>Not found</v>
+        <v>#1, #2</v>
       </c>
       <c r="E5" t="str">
-        <v>Not found</v>
+        <v>N/A</v>
       </c>
       <c r="F5" t="str">
-        <v>zillow.com</v>
+        <v>lianejamason.com</v>
       </c>
     </row>
     <row r="6">
@@ -847,19 +847,19 @@
         <v>2</v>
       </c>
       <c r="B6" t="str">
-        <v>primary keyword 2</v>
+        <v>Corcoran Dwellings St Petersburg</v>
       </c>
       <c r="C6" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="D6" t="str">
-        <v>Not found</v>
+        <v>#4</v>
       </c>
       <c r="E6" t="str">
-        <v>#6</v>
+        <v>N/A</v>
       </c>
       <c r="F6" t="str">
-        <v>example.com</v>
+        <v>corcoran.com</v>
       </c>
     </row>
     <row r="7">
@@ -867,10 +867,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>primary keyword 3</v>
+        <v>St Petersburg FL homes for sale</v>
       </c>
       <c r="C7" t="str">
-        <v>High</v>
+        <v>Very High</v>
       </c>
       <c r="D7" t="str">
         <v>Not found</v>
@@ -879,7 +879,7 @@
         <v>Not found</v>
       </c>
       <c r="F7" t="str">
-        <v>example.com</v>
+        <v>zillow.com</v>
       </c>
     </row>
     <row r="8">
@@ -887,10 +887,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="str">
-        <v>primary keyword 4</v>
+        <v>St Petersburg FL real estate</v>
       </c>
       <c r="C8" t="str">
-        <v>Medium</v>
+        <v>Very High</v>
       </c>
       <c r="D8" t="str">
         <v>Not found</v>
@@ -899,7 +899,7 @@
         <v>Not found</v>
       </c>
       <c r="F8" t="str">
-        <v>example.com</v>
+        <v>zillow.com</v>
       </c>
     </row>
     <row r="9">
@@ -907,31 +907,431 @@
         <v>5</v>
       </c>
       <c r="B9" t="str">
-        <v>primary keyword 5</v>
+        <v>Tampa Bay waterfront homes for sale</v>
       </c>
       <c r="C9" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="D9" t="str">
         <v>Not found</v>
       </c>
       <c r="E9" t="str">
-        <v>#3</v>
+        <v>Not found</v>
       </c>
       <c r="F9" t="str">
-        <v>example.com</v>
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="str">
+        <v>St Pete Beach homes for sale</v>
+      </c>
+      <c r="C10" t="str">
+        <v>High</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F10" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Pinellas County real estate</v>
+      </c>
+      <c r="C11" t="str">
+        <v>High</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F11" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Shore Acres St Petersburg homes for sale</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F12" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Snell Isle homes for sale</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F13" t="str">
+        <v>premiersothebysrealty.com</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Tierra Verde homes for sale</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F14" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>11</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Downtown St Pete condos for sale</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F15" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>12</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Old Northeast St Petersburg real estate</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F16" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17" t="str">
+        <v>buy a home in St Petersburg FL</v>
+      </c>
+      <c r="C17" t="str">
+        <v>High</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F17" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="B18" t="str">
+        <v>sell my house St Petersburg FL</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F18" t="str">
+        <v>stpetefasthomebuyer.com</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>15</v>
+      </c>
+      <c r="B19" t="str">
+        <v>St Petersburg FL real estate agent</v>
+      </c>
+      <c r="C19" t="str">
+        <v>High</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F19" t="str">
+        <v>zillow.com (agent directory)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>16</v>
+      </c>
+      <c r="B20" t="str">
+        <v>best realtor in St Petersburg FL</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Avalon Group ranks</v>
+      </c>
+      <c r="F20" t="str">
+        <v>realestate.usnews.com</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>17</v>
+      </c>
+      <c r="B21" t="str">
+        <v>St Petersburg FL housing market 2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F21" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>18</v>
+      </c>
+      <c r="B22" t="str">
+        <v>luxury homes St Petersburg FL</v>
+      </c>
+      <c r="C22" t="str">
+        <v>High</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E22" t="str">
+        <v>stpetersburgrealestate.com ranks</v>
+      </c>
+      <c r="F22" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>19</v>
+      </c>
+      <c r="B23" t="str">
+        <v>waterfront homes St Petersburg FL</v>
+      </c>
+      <c r="C23" t="str">
+        <v>High</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E23" t="str">
+        <v>stpetersburgrealestate.com, smithandassociates.com rank</v>
+      </c>
+      <c r="F23" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>20</v>
+      </c>
+      <c r="B24" t="str">
+        <v>St Petersburg FL homes with pool</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F24" t="str">
+        <v>redfin.com</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>21</v>
+      </c>
+      <c r="B25" t="str">
+        <v>historic homes St Petersburg FL</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E25" t="str">
+        <v>smithandassociates.com ranks</v>
+      </c>
+      <c r="F25" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>22</v>
+      </c>
+      <c r="B26" t="str">
+        <v>St Pete waterfront condos for sale</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E26" t="str">
+        <v>mygulfcoastproperty.com ranks</v>
+      </c>
+      <c r="F26" t="str">
+        <v>homes.com</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>23</v>
+      </c>
+      <c r="B27" t="str">
+        <v>affordable homes St Petersburg FL</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F27" t="str">
+        <v>homes.com</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>24</v>
+      </c>
+      <c r="B28" t="str">
+        <v>new construction homes St Petersburg FL</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F28" t="str">
+        <v>zillow.com</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>25</v>
+      </c>
+      <c r="B29" t="str">
+        <v>St Petersburg FL investment property</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Not found</v>
+      </c>
+      <c r="F29" t="str">
+        <v>redfin.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G11"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -966,116 +1366,170 @@
         <v>Metric</v>
       </c>
       <c r="B3" t="str">
-        <v>example.com</v>
+        <v>lianejamason.com</v>
       </c>
       <c r="C3" t="str">
-        <v>Competitor 1</v>
+        <v>Avalon Group</v>
       </c>
       <c r="D3" t="str">
-        <v>Competitor 2</v>
+        <v>Eagan Luxury</v>
       </c>
       <c r="E3" t="str">
-        <v>Competitor 3</v>
+        <v>Smith &amp; Associates</v>
       </c>
       <c r="F3" t="str">
-        <v>Competitor 4</v>
+        <v>The Salamone Group</v>
+      </c>
+      <c r="G3" t="str">
+        <v>The Dynasty Group</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Total Pages</v>
+        <v>Blog Posts</v>
       </c>
       <c r="B4" t="str">
-        <v>62</v>
+        <v>287</v>
       </c>
       <c r="C4" t="str">
-        <v>372</v>
+        <v>235</v>
       </c>
       <c r="D4" t="str">
-        <v>376</v>
+        <v>226</v>
       </c>
       <c r="E4" t="str">
-        <v>6x behind</v>
+        <v>Liane leads in volume</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Blog Posts</v>
+        <v>Total Pages</v>
       </c>
       <c r="B5" t="str">
-        <v>5</v>
+        <v>365+</v>
       </c>
       <c r="C5" t="str">
-        <v>96</v>
+        <v>287</v>
       </c>
       <c r="D5" t="str">
-        <v>33</v>
+        <v>381</v>
       </c>
       <c r="E5" t="str">
-        <v>19x behind</v>
+        <v>Mid-range overall</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Key Page Depth</v>
+        <v>Neighborhood Pages</v>
       </c>
       <c r="B6" t="str">
-        <v>~200 words</v>
+        <v>15+</v>
       </c>
       <c r="C6" t="str">
-        <v>500-2,000</v>
+        <v>11</v>
       </c>
       <c r="D6" t="str">
-        <v>3,500-4,500</v>
+        <v>30</v>
       </c>
       <c r="E6" t="str">
-        <v>20x behind</v>
+        <v>Behind Eagan &amp; Smith</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Schema Markup</v>
+        <v>Homepage Meta Desc</v>
       </c>
       <c r="B7" t="str">
-        <v>None</v>
+        <v>MISSING</v>
       </c>
       <c r="C7" t="str">
-        <v>None</v>
+        <v>Present</v>
       </c>
       <c r="D7" t="str">
-        <v>Yes</v>
+        <v>Present</v>
       </c>
       <c r="E7" t="str">
-        <v>Missing</v>
+        <v>Critical gap</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Keywords Ranking</v>
+        <v>Schema Depth</v>
       </c>
       <c r="B8" t="str">
-        <v>0 / 25</v>
+        <v>Moderate</v>
       </c>
       <c r="C8" t="str">
-        <v>5 / 25</v>
+        <v>Moderate</v>
       </c>
       <c r="D8" t="str">
-        <v>12 / 25</v>
+        <v>Excellent</v>
       </c>
       <c r="E8" t="str">
-        <v>Zero visibility</v>
+        <v>Behind Eagan Luxury</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Reviews Highlighted</v>
+      </c>
+      <c r="B9" t="str">
+        <v>"Top 3" badge</v>
+      </c>
+      <c r="C9" t="str">
+        <v>300+ 5-star</v>
+      </c>
+      <c r="D9" t="str">
+        <v>85, 5.0 stars</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Under-leveraged</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Lead Magnets</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Broken home value form</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Reports, guides, SMS</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Valuation, consultation</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Zero functional magnets</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Est. Domain Rating</v>
+      </c>
+      <c r="B11" t="str">
+        <v>20-30</v>
+      </c>
+      <c r="C11" t="str">
+        <v>35-45</v>
+      </c>
+      <c r="D11" t="str">
+        <v>30-40</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Below top competitors</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E58"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -1140,16 +1594,16 @@
         <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>Fix broken/error pages — remove from sitemap, add noindex</v>
+        <v>Fix Market Analysis page form — broken lead capture</v>
       </c>
       <c r="C5" t="str">
-        <v>Broken pages waste crawl budget</v>
+        <v>Primary seller lead page is a dead end; every homepage CTA leads here</v>
       </c>
       <c r="D5" t="str">
         <v>Low</v>
       </c>
       <c r="E5" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
     </row>
     <row r="6">
@@ -1157,10 +1611,10 @@
         <v>2</v>
       </c>
       <c r="B6" t="str">
-        <v>Fix corrupted meta tags</v>
+        <v>Write meta descriptions for all core pages missing them</v>
       </c>
       <c r="C6" t="str">
-        <v>Bad meta tags look spammy to Google</v>
+        <v>60%+ of core pages have no meta descriptions; Google auto-generates poor snippets</v>
       </c>
       <c r="D6" t="str">
         <v>Low</v>
@@ -1174,10 +1628,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Consolidate to single H1 per page</v>
+        <v>Rewrite homepage title tag to front-load keywords</v>
       </c>
       <c r="C7" t="str">
-        <v>Multiple H1s dilute topic signal</v>
+        <v>'Home - Liane Jamason' wastes the most valuable on-page ranking element</v>
       </c>
       <c r="D7" t="str">
         <v>Low</v>
@@ -1191,16 +1645,16 @@
         <v>4</v>
       </c>
       <c r="B8" t="str">
-        <v>Rewrite meta descriptions with location keywords</v>
+        <v>Fix Active Listings meta (says 'View My Sold Listings')</v>
       </c>
       <c r="C8" t="str">
-        <v>Generic descriptions provide zero advantage</v>
+        <v>Describes the wrong page — confuses users and search engines</v>
       </c>
       <c r="D8" t="str">
         <v>Low</v>
       </c>
       <c r="E8" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="9">
@@ -1208,10 +1662,10 @@
         <v>5</v>
       </c>
       <c r="B9" t="str">
-        <v>Add Open Graph tags</v>
+        <v>Noindex off-topic pages (travel hacking, credit card points)</v>
       </c>
       <c r="C9" t="str">
-        <v>Social shares display poorly without OG tags</v>
+        <v>Off-topic content dilutes topical authority; penalized by March 2026 core update</v>
       </c>
       <c r="D9" t="str">
         <v>Low</v>
@@ -1225,16 +1679,16 @@
         <v>6</v>
       </c>
       <c r="B10" t="str">
-        <v>Add canonical tags to dynamic pages</v>
+        <v>Disable attachment page indexing in Rank Math</v>
       </c>
       <c r="C10" t="str">
-        <v>Missing canonicals cause duplicate content issues</v>
+        <v>7 attachment sitemaps feeding hundreds of thin pages into Google's index</v>
       </c>
       <c r="D10" t="str">
         <v>Low</v>
       </c>
       <c r="E10" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
     </row>
     <row r="11">
@@ -1242,101 +1696,101 @@
         <v>7</v>
       </c>
       <c r="B11" t="str">
-        <v>Add LocalBusiness + industry schema to key pages</v>
+        <v>Fix or remove broken idx_page-sitemap.xml</v>
       </c>
       <c r="C11" t="str">
-        <v>Schema enables rich results in Google</v>
+        <v>Broken sitemap (404) signals poor maintenance to Google</v>
       </c>
       <c r="D11" t="str">
         <v>Low</v>
       </c>
       <c r="E11" t="str">
-        <v>High</v>
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Update StPetersburg.com listing (still shows Smith &amp; Associates)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Outdated citation with wrong brokerage affiliation hurts local SEO</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Claim Yelp, Realtor.com, Redfin, BBB, Bing Places profiles</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Missing from DA 90+ directories where all competitors are present</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E13" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Fix Market Analysis meta description typo ('you home' → 'your home')</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Typo in the most important seller lead page meta tag</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Low</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>SHORT-TERM — Month 1-2 (Medium Effort)</v>
       </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>#</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B17" t="str">
         <v>Action</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C17" t="str">
         <v>Why</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D17" t="str">
         <v>Effort</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E17" t="str">
         <v>Impact</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>8</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Write and publish market/industry report with current data</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Top content type for this industry's SEO</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="E15" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>9</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Expand top 10 key pages from thin to 1,000-1,500 words</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Thin pages can't compete; competitors have 2,000+</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="E16" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>10</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Write 4-6 new locally-focused blog posts</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Fresh local content essential for rankings</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="E17" t="str">
-        <v>High</v>
       </c>
     </row>
     <row r="18">
@@ -1344,10 +1798,10 @@
         <v>11</v>
       </c>
       <c r="B18" t="str">
-        <v>Add contact forms + CTAs to every key page</v>
+        <v>Fix all H1 tag issues (duplicates on 8+ pages, missing on blog index, generic on 5+ pages)</v>
       </c>
       <c r="C18" t="str">
-        <v>Best pages have no conversion mechanism</v>
+        <v>H1 is the primary on-page topic signal; violations on critical pages</v>
       </c>
       <c r="D18" t="str">
         <v>Low</v>
@@ -1361,16 +1815,16 @@
         <v>12</v>
       </c>
       <c r="B19" t="str">
-        <v>Create testimonials/reviews page</v>
+        <v>Rewrite all core page title tags (About, Sell, Buy, Contact, Blog)</v>
       </c>
       <c r="C19" t="str">
-        <v>Builds trust; every competitor has one</v>
+        <v>Generic titles waste ranking potential; competitors front-load keywords</v>
       </c>
       <c r="D19" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="E19" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
     </row>
     <row r="20">
@@ -1378,81 +1832,98 @@
         <v>13</v>
       </c>
       <c r="B20" t="str">
-        <v>Rewrite About page with credentials and video</v>
+        <v>Update Buy page to remove 'Jamason Group' branding</v>
       </c>
       <c r="C20" t="str">
-        <v>Current version doesn't sell expertise</v>
+        <v>Old branding confuses users and search engines</v>
       </c>
       <c r="D20" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="E20" t="str">
         <v>Medium</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21">
+        <v>14</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Add email newsletter signup to blog sidebar and post footers</v>
+      </c>
+      <c r="C21" t="str">
+        <v>287 blog posts generating zero email subscribers — biggest conversion gap</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E21" t="str">
+        <v>High</v>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" t="str">
-        <v>MEDIUM-TERM — Month 2-4 (Higher Effort)</v>
+      <c r="A22">
+        <v>15</v>
       </c>
       <c r="B22" t="str">
-        <v/>
+        <v>Add end-of-post CTAs to all blog articles</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>High-value content like '9 Mistakes' article has no conversion path</v>
       </c>
       <c r="D22" t="str">
-        <v/>
+        <v>Medium</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>High</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="str">
-        <v>#</v>
+      <c r="A23">
+        <v>16</v>
       </c>
       <c r="B23" t="str">
-        <v>Action</v>
+        <v>Rewrite Sell page with real seller content, process, and CTAs</v>
       </c>
       <c r="C23" t="str">
-        <v>Why</v>
+        <v>Current page is a testimonial wall with ~150 words and no lead capture</v>
       </c>
       <c r="D23" t="str">
-        <v>Effort</v>
+        <v>Medium</v>
       </c>
       <c r="E23" t="str">
-        <v>Impact</v>
+        <v>High</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B24" t="str">
-        <v>Create comprehensive hub page for top keyword cluster</v>
+        <v>Add alt text to all content images (hero, headshot, press logos, property photos)</v>
       </c>
       <c r="C24" t="str">
-        <v>Top competitor has hub + sub-pages for this topic</v>
+        <v>70-83% missing; hurts accessibility, image search, and AI understanding</v>
       </c>
       <c r="D24" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E24" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B25" t="str">
-        <v>Create topical section pages (e.g. /topic/)</v>
+        <v>Fix broken pages (In the Press, Short Sales, Clearwater)</v>
       </c>
       <c r="C25" t="str">
-        <v>Competitors have 20+ pages per topic vs. client's 1</v>
+        <v>Pages that timeout are invisible to both users and Googlebot; Press page has strongest E-E-A-T signals</v>
       </c>
       <c r="D25" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E25" t="str">
         <v>High</v>
@@ -1460,16 +1931,16 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B26" t="str">
-        <v>Create relocation/moving guide (2,000+ words)</v>
+        <v>Add AggregateRating/Review schema to Reviews page</v>
       </c>
       <c r="C26" t="str">
-        <v>High-value informational keyword</v>
+        <v>Enables star ratings in SERPs; 90+ reviews = strong social proof being wasted</v>
       </c>
       <c r="D26" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E26" t="str">
         <v>High</v>
@@ -1477,98 +1948,98 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B27" t="str">
-        <v>Build sub-pages for top 20 listings/locations/products</v>
+        <v>Verify/optimize Google Business Profile; begin weekly posting</v>
       </c>
       <c r="C27" t="str">
-        <v>Top competitor has 150+ individual pages</v>
+        <v>GBP accounts for 30%+ of map pack visibility; AI Overviews pull from GBP</v>
       </c>
       <c r="D27" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="E27" t="str">
         <v>High</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28">
-        <v>18</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Add FAQ sections with schema to all key pages</v>
-      </c>
-      <c r="C28" t="str">
-        <v>FAQ schema generates rich snippets + AI citations</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="E28" t="str">
-        <v>High</v>
-      </c>
-    </row>
     <row r="29">
-      <c r="A29">
-        <v>19</v>
+      <c r="A29" t="str">
+        <v>MEDIUM-TERM — Month 2-4 (Higher Effort)</v>
       </c>
       <c r="B29" t="str">
-        <v>Implement cross-linking strategy across all content</v>
+        <v/>
       </c>
       <c r="C29" t="str">
-        <v>Competitors link everything; client relies on nav only</v>
+        <v/>
       </c>
       <c r="D29" t="str">
-        <v>Medium</v>
+        <v/>
       </c>
       <c r="E29" t="str">
-        <v>Medium</v>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>#</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Action</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Why</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Effort</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Impact</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="str">
-        <v>LONG-TERM — Month 4+ (Ongoing Strategy)</v>
+      <c r="A31">
+        <v>21</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>Create 7 neighborhood landing pages (Snell Isle, Old NE, Downtown, Shore Acres, Tierra Verde, Venetian Isles, Coffee Pot Bayou)</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>Neighborhood queries have lowest portal density and highest local opportunity</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>High</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>Very High</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="str">
-        <v>#</v>
+      <c r="A32">
+        <v>22</v>
       </c>
       <c r="B32" t="str">
-        <v>Action</v>
+        <v>Create 5 property-type landing pages (Waterfront Homes, Luxury Homes, Waterfront Condos, Downtown Condos, Historic Homes)</v>
       </c>
       <c r="C32" t="str">
-        <v>Why</v>
+        <v>Critical keyword gaps directly aligned with core services; competitors have dedicated pages</v>
       </c>
       <c r="D32" t="str">
-        <v>Effort</v>
+        <v>High</v>
       </c>
       <c r="E32" t="str">
-        <v>Impact</v>
+        <v>Very High</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B33" t="str">
-        <v>Monthly report publishing cadence</v>
+        <v>Expand existing top neighborhood pages to 2,000+ words with market stats</v>
       </c>
       <c r="C33" t="str">
-        <v>Consistency builds authority</v>
+        <v>Current pages are 250-550 words; 2026 benchmark is 2,000-3,000</v>
       </c>
       <c r="D33" t="str">
         <v>Medium</v>
@@ -1579,16 +2050,16 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B34" t="str">
-        <v>Build content library toward 200+ pages</v>
+        <v>Add FAQPage schema to blog posts with FAQ sections</v>
       </c>
       <c r="C34" t="str">
-        <v>Minimum to compete for topical authority</v>
+        <v>Earns rich results in SERPs; high AI citation value for Market Update, Best Neighborhoods</v>
       </c>
       <c r="D34" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E34" t="str">
         <v>High</v>
@@ -1596,13 +2067,13 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B35" t="str">
-        <v>Create lifestyle/resource content</v>
+        <v>Implement BreadcrumbList schema site-wide</v>
       </c>
       <c r="C35" t="str">
-        <v>Attracts traffic that builds domain authority</v>
+        <v>Improves navigation for users and search engines; enables breadcrumb rich results</v>
       </c>
       <c r="D35" t="str">
         <v>Medium</v>
@@ -1613,33 +2084,33 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B36" t="str">
-        <v>Create comparison content (vs. competitors/alternatives)</v>
+        <v>Join St. Petersburg Chamber of Commerce</v>
       </c>
       <c r="C36" t="str">
-        <v>Attracts buyers comparing options</v>
+        <v>Networking + DA 45 backlink from business.stpete.com; Smith &amp; Associates is a confirmed member</v>
       </c>
       <c r="D36" t="str">
         <v>Medium</v>
       </c>
       <c r="E36" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B37" t="str">
-        <v>Video content series</v>
+        <v>Contact Johns Hopkins All Children's Hospital for donor page backlink</v>
       </c>
       <c r="C37" t="str">
-        <v>Video builds trust; embed on pages + YouTube</v>
+        <v>$25K donation generating zero link equity; .org backlink from prestigious institution</v>
       </c>
       <c r="D37" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E37" t="str">
         <v>High</v>
@@ -1647,13 +2118,13 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B38" t="str">
-        <v>Build local citations and profiles</v>
+        <v>Create 'Moving to St. Petersburg' relocation guide (2,000+ words)</v>
       </c>
       <c r="C38" t="str">
-        <v>Strengthens map-pack/local visibility</v>
+        <v>High-volume keyword opportunity; no current content for relocating buyers</v>
       </c>
       <c r="D38" t="str">
         <v>Medium</v>
@@ -1664,24 +2135,330 @@
     </row>
     <row r="39">
       <c r="A39">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B39" t="str">
-        <v>Email newsletter with regular updates</v>
+        <v>Create a downloadable lead magnet (Waterfront Buyer's Checklist or Market Report PDF)</v>
       </c>
       <c r="C39" t="str">
-        <v>Email converts higher than any other channel</v>
+        <v>Competitors offer 2+ downloadable guides; Liane offers zero</v>
       </c>
       <c r="D39" t="str">
         <v>Medium</v>
       </c>
       <c r="E39" t="str">
         <v>High</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>30</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Reduce script/stylesheet bloat; audit unused plugins</v>
+      </c>
+      <c r="C40" t="str">
+        <v>36-63 scripts per page impacting Core Web Vitals; About page loads 61 scripts, 17 stylesheets</v>
+      </c>
+      <c r="D40" t="str">
+        <v>High</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>31</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Consolidate phone numbers to one number across all pages</v>
+      </c>
+      <c r="C41" t="str">
+        <v>3 different numbers (727-755-3325, 727-240-3636, 727-888-HOME) hurts local SEO</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>32</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Fix schema types (Homepage to WebPage, About to AboutPage, change author 'varick' to Liane)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Incorrect schema types reduce trust signals and AI citation likelihood</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>33</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Add 'Notable Sales' section to homepage or dedicated page</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Dynasty Group shows specific $14M, $13M sales — far more compelling than 'Top 1%' claims</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>LONG-TERM — Month 4+ (Ongoing Strategy)</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>#</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Action</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Why</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Effort</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Impact</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>34</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Publish monthly 'St. Petersburg Waterfront Market Report' with proprietary data</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Original data studies show 22% visibility increase; serves as content marketing and link bait</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Very High</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>35</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Build 10+ additional neighborhood pages (Clearwater, Gulfport, Tampa, Kenwood, Crescent Lake)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Expand geographic coverage; fill content gaps for areas with 0-50 words currently</v>
+      </c>
+      <c r="D48" t="str">
+        <v>High</v>
+      </c>
+      <c r="E48" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>36</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Create condo building pages (Waldorf Astoria, Saltaire, ONE St Pete, 400 Central, The Salvador)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Eagan dominates with 20+ pages; high-intent '[building name] condos' keywords</v>
+      </c>
+      <c r="D49" t="str">
+        <v>High</v>
+      </c>
+      <c r="E49" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>37</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Pitch Tampa Bay Times for recurring column or expert feature</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Already has relationship (multiple past quotes); high-authority editorial backlink</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Very High</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>38</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Re-engage national press contacts via HARO/Connectively</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Reactivate Forbes, WSJ, USA Today relationships; earn ongoing DA 80+ citations</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E51" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>39</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Guest post on St Pete Catalyst, Tampa Real Estate Insider, I Love the Burg</v>
+      </c>
+      <c r="C52" t="str">
+        <v>DA 50+ editorial backlinks from locally relevant publications</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>40</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Create video content hub on site with YouTube embeds + VideoObject schema</v>
+      </c>
+      <c r="C53" t="str">
+        <v>9+ TV segments and YouTube channel not leveraged on site; video carousels in SERPs</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>41</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Build lifestyle content hub (restaurants, events, local guides per neighborhood)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Avalon and Salamone Group drive significant traffic with this content type</v>
+      </c>
+      <c r="D54" t="str">
+        <v>High</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>42</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Develop school district guide and neighborhood comparison tool</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Key buyer decision factors missing from site; competitors cover these</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>43</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Partner with USF St. Petersburg for guest lectures / internships (.edu backlink)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>DA 80+ .edu backlink; real estate program recently received $1.25M gift</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E56" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>44</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Sponsor local events (SHINE Mural Festival, Localtopia, Habitat for Humanity gala)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Backlinks from .org event pages + community visibility</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>45</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Evaluate site redesign / theme modernization</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Genesis/AgentPress theme is functional but dated vs. Eagan's modern stack and Dynasty's Luxury Presence site</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Very High</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Medium</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1712,7 +2489,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Month 1: Establish Credibility</v>
+        <v>Month 1: Establish Market Authority</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -1743,13 +2520,13 @@
         <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>Industry/Market Report: Current Data</v>
+        <v>St. Petersburg Housing Market Update: Spring 2026</v>
       </c>
       <c r="C5" t="str">
-        <v>primary market keyword</v>
+        <v>st petersburg fl housing market 2026</v>
       </c>
       <c r="D5" t="str">
-        <v>Market Report</v>
+        <v>Market Update</v>
       </c>
     </row>
     <row r="6">
@@ -1757,13 +2534,13 @@
         <v>2</v>
       </c>
       <c r="B6" t="str">
-        <v>Best [Locations/Options] Guide (Current Year)</v>
+        <v>The Complete Guide to Buying a Waterfront Home in St. Petersburg</v>
       </c>
       <c r="C6" t="str">
-        <v>best locations keyword</v>
+        <v>waterfront homes st petersburg fl</v>
       </c>
       <c r="D6" t="str">
-        <v>Guide</v>
+        <v>Pillar / Evergreen</v>
       </c>
     </row>
     <row r="7">
@@ -1771,13 +2548,13 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Is [Industry] a Good Investment?</v>
+        <v>Snell Isle: St. Petersburg's Premier Waterfront Community</v>
       </c>
       <c r="C7" t="str">
-        <v>investment keyword</v>
+        <v>snell isle homes for sale</v>
       </c>
       <c r="D7" t="str">
-        <v>Informational</v>
+        <v>Neighborhood Deep-Dive</v>
       </c>
     </row>
     <row r="8">
@@ -1785,18 +2562,18 @@
         <v>4</v>
       </c>
       <c r="B8" t="str">
-        <v>Major Development/Trend: What Buyers Need to Know</v>
+        <v>Is Now a Good Time to Buy a Home in St. Petersburg FL? (2026 Analysis)</v>
       </c>
       <c r="C8" t="str">
-        <v>trend keyword</v>
+        <v>buy a home in st petersburg fl</v>
       </c>
       <c r="D8" t="str">
-        <v>News/Analysis</v>
+        <v>Informational / FAQ</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Month 2: Build Depth</v>
+        <v>Month 2: Build Neighborhood Depth</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -1827,13 +2604,13 @@
         <v>1</v>
       </c>
       <c r="B12" t="str">
-        <v>Relocation/Getting Started Guide</v>
+        <v>Best Neighborhoods in St. Petersburg FL for Waterfront Living</v>
       </c>
       <c r="C12" t="str">
-        <v>relocation keyword</v>
+        <v>waterfront homes st petersburg fl</v>
       </c>
       <c r="D12" t="str">
-        <v>Guide</v>
+        <v>Comparison / Pillar</v>
       </c>
     </row>
     <row r="13">
@@ -1841,13 +2618,13 @@
         <v>2</v>
       </c>
       <c r="B13" t="str">
-        <v>Premium/Specialty Offering Guide</v>
+        <v>What to Know About Flood Insurance for St. Petersburg Waterfront Homes</v>
       </c>
       <c r="C13" t="str">
-        <v>specialty keyword</v>
+        <v>waterfront home flood insurance florida</v>
       </c>
       <c r="D13" t="str">
-        <v>Property Guide</v>
+        <v>Expert / E-E-A-T</v>
       </c>
     </row>
     <row r="14">
@@ -1855,13 +2632,13 @@
         <v>3</v>
       </c>
       <c r="B14" t="str">
-        <v>Comparison: Your Market vs. Alternative</v>
+        <v>Historic Old Northeast: Architecture, Lifestyle &amp; Real Estate Guide</v>
       </c>
       <c r="C14" t="str">
-        <v>comparison keyword</v>
+        <v>old northeast st petersburg real estate</v>
       </c>
       <c r="D14" t="str">
-        <v>Comparison</v>
+        <v>Neighborhood Deep-Dive</v>
       </c>
     </row>
     <row r="15">
@@ -1869,18 +2646,18 @@
         <v>4</v>
       </c>
       <c r="B15" t="str">
-        <v>Costs, Fees, and Practical FAQ</v>
+        <v>Selling Your St. Petersburg Home in 2026: The Complete Guide</v>
       </c>
       <c r="C15" t="str">
-        <v>practical keyword</v>
+        <v>sell my house st petersburg fl</v>
       </c>
       <c r="D15" t="str">
-        <v>FAQ/Guide</v>
+        <v>Seller Resource / Pillar</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Month 3: Expand Reach</v>
+        <v>Month 3: Expand Reach &amp; Convert</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -1911,13 +2688,13 @@
         <v>1</v>
       </c>
       <c r="B19" t="str">
-        <v>Quarterly Market Update</v>
+        <v>Downtown St. Pete Condo Market Report: Prices, Inventory &amp; Outlook</v>
       </c>
       <c r="C19" t="str">
-        <v>market update keyword</v>
+        <v>downtown st pete condos for sale</v>
       </c>
       <c r="D19" t="str">
-        <v>Market Report</v>
+        <v>Market Update / Data</v>
       </c>
     </row>
     <row r="20">
@@ -1925,13 +2702,13 @@
         <v>2</v>
       </c>
       <c r="B20" t="str">
-        <v>Adjacent Area/Hidden Gem Guide</v>
+        <v>Shore Acres vs. Old Northeast: Which Neighborhood Is Right for You?</v>
       </c>
       <c r="C20" t="str">
-        <v>adjacent area keyword</v>
+        <v>shore acres st petersburg homes for sale</v>
       </c>
       <c r="D20" t="str">
-        <v>Area Guide</v>
+        <v>Comparison</v>
       </c>
     </row>
     <row r="21">
@@ -1939,13 +2716,13 @@
         <v>3</v>
       </c>
       <c r="B21" t="str">
-        <v>Regulations/Rules Investors Need to Know</v>
+        <v>Moving to St. Petersburg FL: The Complete Relocation Guide</v>
       </c>
       <c r="C21" t="str">
-        <v>regulations keyword</v>
+        <v>moving to st petersburg fl</v>
       </c>
       <c r="D21" t="str">
-        <v>Investment Guide</v>
+        <v>Pillar / Evergreen</v>
       </c>
     </row>
     <row r="22">
@@ -1953,13 +2730,13 @@
         <v>4</v>
       </c>
       <c r="B22" t="str">
-        <v>Luxury/Premium Segment Deep Dive</v>
+        <v>St. Petersburg Real Estate Investment: Cap Rates, Rental Markets &amp; Opportunity Zones</v>
       </c>
       <c r="C22" t="str">
-        <v>luxury keyword</v>
+        <v>st petersburg fl investment property</v>
       </c>
       <c r="D22" t="str">
-        <v>Luxury Guide</v>
+        <v>Investor-Focused</v>
       </c>
     </row>
   </sheetData>
@@ -2026,13 +2803,13 @@
         <v>Meta Titles &amp; Descriptions</v>
       </c>
       <c r="B5" t="str">
-        <v>All pages</v>
+        <v>20+ pages (core, neighborhood, blog, utility)</v>
       </c>
       <c r="C5" t="str">
-        <v>8.75/10</v>
+        <v>9.00/10</v>
       </c>
       <c r="D5" t="str">
-        <v>Ready — verify claims with client</v>
+        <v>Ready — 2 versions created (Claude + Codex), verify URLs and paste into Rank Math</v>
       </c>
     </row>
     <row r="6">
@@ -2040,27 +2817,27 @@
         <v>Schema Markup (JSON-LD)</v>
       </c>
       <c r="B6" t="str">
-        <v>8 schema blocks</v>
+        <v>8+ schema blocks (Organization, RealEstateAgent, AggregateRating, FAQPage, BreadcrumbList, AboutPage, Service, WebSite)</v>
       </c>
       <c r="C6" t="str">
         <v>9.00/10</v>
       </c>
       <c r="D6" t="str">
-        <v>Ready — verify URLs</v>
+        <v>Ready — 2 versions created, verify license number and review count before deploying</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Key Pages (expanded content)</v>
+        <v>Community/Neighborhood Pages</v>
       </c>
       <c r="B7" t="str">
-        <v>4 pages, 1,000+ words</v>
+        <v>Downtown St Pete Condos + additional neighborhoods (2,000+ words each)</v>
       </c>
       <c r="C7" t="str">
         <v>8.75/10</v>
       </c>
       <c r="D7" t="str">
-        <v>Ready — paste into CMS</v>
+        <v>Ready — 2 versions created, paste into CMS as new pages</v>
       </c>
     </row>
     <row r="8">
@@ -2068,13 +2845,13 @@
         <v>Blog Posts (SEO-optimized)</v>
       </c>
       <c r="B8" t="str">
-        <v>4 posts, 900-1,200 words</v>
+        <v>4 posts: Market Report, Waterfront Guide, Snell Isle Deep-Dive, Is Now a Good Time to Buy</v>
       </c>
       <c r="C8" t="str">
         <v>9.00/10</v>
       </c>
       <c r="D8" t="str">
-        <v>Ready — paste into CMS</v>
+        <v>Ready — 2 versions created, paste into WordPress blog</v>
       </c>
     </row>
     <row r="10">
@@ -2096,7 +2873,7 @@
         <v>1</v>
       </c>
       <c r="B11" t="str">
-        <v>Page 1</v>
+        <v>Downtown St. Pete Condos for Sale</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -2110,7 +2887,7 @@
         <v>2</v>
       </c>
       <c r="B12" t="str">
-        <v>Page 2</v>
+        <v>St. Petersburg Waterfront Homes Guide</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -2124,7 +2901,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="str">
-        <v>Page 3</v>
+        <v>Snell Isle Neighborhood Deep-Dive</v>
       </c>
       <c r="C13" t="str">
         <v/>
@@ -2138,7 +2915,7 @@
         <v>4</v>
       </c>
       <c r="B14" t="str">
-        <v>Page 4</v>
+        <v>Selling Your St. Petersburg Home Guide</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -2166,7 +2943,7 @@
         <v>1</v>
       </c>
       <c r="B17" t="str">
-        <v>Blog Post 1</v>
+        <v>St. Petersburg FL Real Estate Market Report: Spring 2026</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -2180,7 +2957,7 @@
         <v>2</v>
       </c>
       <c r="B18" t="str">
-        <v>Blog Post 2</v>
+        <v>The Complete Guide to Buying a Waterfront Home in St. Petersburg</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -2194,7 +2971,7 @@
         <v>3</v>
       </c>
       <c r="B19" t="str">
-        <v>Blog Post 3</v>
+        <v>Snell Isle: St. Petersburg's Premier Waterfront Community</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -2208,7 +2985,7 @@
         <v>4</v>
       </c>
       <c r="B20" t="str">
-        <v>Blog Post 4</v>
+        <v>Is Now a Good Time to Buy a Home in St. Petersburg FL?</v>
       </c>
       <c r="C20" t="str">
         <v/>

</xml_diff>